<commit_message>
Add SOURCE_SCAN docs, archived EI inputs, and batch explanation outputs.
Canonicalize the Scan ABAP Report Sources input set, archive prior EI workbooks under input/old, and sync pipeline run artifacts plus generated explanations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/input/old/Available fields_SKN_S_SW_10_06_MD_CHNG_LOG.xlsx
+++ b/input/old/Available fields_SKN_S_SW_10_06_MD_CHNG_LOG.xlsx
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Object value</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2761,13 +2761,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Parameters, #of Fields = 21</t>
+          <t>Parameters, #of Fields = 72</t>
         </is>
       </c>
     </row>
@@ -2811,71 +2811,71 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BACKDAYS</t>
+          <t>ACT_CHNGNO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Backdays</t>
+          <t>Document number</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CD_CHNGNO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CDCHANGENR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CHANGENR</t>
+          <t>BACKDAYS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Document number</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CHAR</t>
+          <t>Backdays</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>CDCHANGENR</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>CDCHANGENR</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHANGE_IND</t>
+          <t>CHANGENR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Appl. object change-Header Lvl</t>
+          <t>Document number</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2895,24 +2895,24 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CDCHNGINDH</t>
+          <t>CDCHANGENR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CDCHNGIND</t>
+          <t>CDCHANGENR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHNGIND</t>
+          <t>CHANGE_IND</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Change Indicator-Row lvl</t>
+          <t>Appl. object change-Header Lvl</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CDCHNGIND</t>
+          <t>CDCHNGINDH</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2944,134 +2944,224 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CONVERT_KEY</t>
+          <t>CHANGE_IND_DESC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>'X' - Decompose Key Field</t>
+          <t>Domain name</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DOMNAME</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DOMNAME</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DATUM</t>
+          <t>CHNGIND</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Change Indicator-Row lvl</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CDCHNGIND</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CDCHNGIND</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DURATION_D</t>
+          <t>CHNGIND_DESC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Domain name</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>DOMNAME</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>DOMNAME</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FNAME</t>
+          <t>CONVERT_KEY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Field Name</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CHAR</t>
+          <t>'X' - Decompose Key Field</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>FIELDNAME</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>FDNAME</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HEADER_ONLY</t>
+          <t>CUKY_NEW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CHAR</t>
+          <t>CUKY</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CUKY</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>XFELD</t>
+          <t>CDCUKY</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>WAERS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LANGU</t>
+          <t>CUKY_OLD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Language for texts</t>
+          <t>CUKY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CUKY</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CDCUKY</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>WAERS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MANAGE_IN_UTC</t>
+          <t>DATUM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>'X' - Manage in UTC</t>
+          <t>DATS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3081,56 +3171,51 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>DATUM</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DATUM</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OBJECTCLAS</t>
+          <t>DURATION_D</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Change doc. object</t>
+          <t>INT4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CHAR</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>CDOBJECTCL</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>OBJECTCL</t>
+          <t>/SKN/E_SW_DURATION_D</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OBJECTID</t>
+          <t>FIELD_DESC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Short Description</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3140,7 +3225,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3150,100 +3235,120 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>CDOBJECTV</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CHAR90</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REPET_BACKDAYS</t>
+          <t>FNAME</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INT4</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>REPETITIVE</t>
+          <t>FNAME_REP</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>'X' - Repetitive Change</t>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHAR</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FIELDNAME</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>/SKN/E_REPEAT</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>XFLAG</t>
+          <t>FDNAME</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SW_DEST</t>
+          <t>HEADER_ONLY</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>XFELD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TABNAME</t>
+          <t>KEY1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Table Name</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3263,24 +3368,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TABNAME</t>
+          <t>FIELDNAME</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>AS4TAB</t>
+          <t>FDNAME</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TCODE</t>
+          <t>KEY1_DS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Transaction Code</t>
+          <t>Short Description</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3290,7 +3395,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3300,34 +3405,34 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CDTCODE</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TCODE</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>UDATE</t>
+          <t>KEY1_V</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Short Description</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DATS</t>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3337,81 +3442,1918 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CDDATUM</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>DATUM</t>
+          <t>AS4TEXT</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>UDATE_REPET</t>
+          <t>KEY2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DATS</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>CHAR</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CDDATUM</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>DATUM</t>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>KEY2_DS</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KEY2_V</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KEY3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KEY3_DS</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KEY3_V</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>KEY4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>KEY4_DS</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>KEY4_V</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>KEY5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>KEY5_DS</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>KEY5_V</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>KEY6</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>KEY6_DS</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>KEY6_V</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>KEY7</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KEY7_DS</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>KEY7_V</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KEY8</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KEY8_DS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KEY8_V</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KEY9</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KEY9_DS</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KEY9_V</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KEY10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>FIELDNAME</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>FDNAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KEY10_DS</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>KEY10_V</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LANGU</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Language for texts</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MANAGE_IN_UTC</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>'X' - Manage in UTC</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>NAME_FIRST</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>First name</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>AD_NAMEFIR</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>TEXT40</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NAME_LAST</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Last name</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>AD_NAMELAS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>TEXT40</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NAME_TEXT</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>AD_NAMTEXT</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>TEXT80</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>OBJECTCLAS</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Change doc. object</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>CDOBJECTCL</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>OBJECTCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>OBJECTID</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>CDOBJECTV</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>CHAR90</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>OBJECT_DESC</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>NAME1_GP</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PLANCHNGNR</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Change number</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>PLANCHNGNR</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>PLANCHNGNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>REPET_BACKDAYS</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>INT4</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>REPETITIVE</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Repetitive Change</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>/SKN/E_REPEAT</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>XFLAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SW_DEST</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>RFCDEST</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>RFCDEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TABKEY</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Table Key</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>CDTABKEY</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>CHAR70</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TABNAME</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Table Name</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TABNAME</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>AS4TAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TAB_DESC</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Short Description</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>AS4TEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TCODE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Transaction Code</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>CDTCODE</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>TCODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TEXT_CASE</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Text flag</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>CDXFELD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>XFELD</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UDATE</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>DATS</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>CDDATUM</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>DATUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>UDATE_REPET</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>DATS</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>CDDATUM</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>DATUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>UNIT_NEW</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CDUNIT</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>CDUNIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>UNIT_OLD</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CDUNIT</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>CDUNIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
           <t>USERNAME</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>CHAR</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>CDUSERNAME</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>CHAR12</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>UTIME</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>TIMS</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>CDUZEIT</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>UZEIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>VALUE_NEW</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>New value</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>CDFLDVALN</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>FIELDVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>VALUE_OLD</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Old value</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>CDFLDVALO</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>FIELDVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>WAS_PLANND</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>gen from plan. changes</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CHAR</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>CD_PLANNED</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>XFLAG</t>
         </is>
       </c>
     </row>

</xml_diff>